<commit_message>
feat: Demo D3 - PrimitiveMesh 渲染 + 分离 AI + 场景优化
Render 层:
- 新增 PrimitiveMeshAgent: 按 ModelInfo.Type/Mesh/Size/Color 程序化生成 Box/Cylinder/Sphere
- 新增 PrimitiveAnimAgent: 按 animstate 做程序化动画 (IDLE/MOVE/BEHIT/DEATH/CASTING)
- ModelEnchant / AnimationEnchant 按 ModelInfo.Type 分叉路由
- World: 注册 PrimitiveMeshAgent.SetRoot, 加棋盘格地面 shader, 压暗场景灯光

Logic 层:
- ChargeAI 加分离力 (separation steering), 避免敌人堆叠

配置:
- ModelInfo 新增 Type/Mesh/Size/Color 四列, 怪物 200001 改为橙色方块

UI:
- 所有按钮/CheckBox 补全 font_pressed_color / font_hover_color, 消除白色状态
- 单位信息标签改用 SpatialAgent.position (插值后), 消除抖动

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Config/Datas/ModelData.xlsx
+++ b/Config/Datas/ModelData.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="17"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="1"/>
@@ -516,6 +516,26 @@
           <t>Animation</t>
         </is>
       </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>Mesh</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="H1" s="0" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -538,6 +558,26 @@
           <t>string</t>
         </is>
       </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>(list#sep=|),int</t>
+        </is>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
+        <is>
+          <t>(list#sep=|),int</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -558,6 +598,26 @@
       <c r="D3" s="7" t="inlineStr">
         <is>
           <t>动画路径</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>类型(glb/primitive)</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>基元形状(box/cylinder/sphere)</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>尺寸(mm)</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>颜色(RGBA 0-255)</t>
         </is>
       </c>
     </row>
@@ -570,27 +630,70 @@
           <t>Hero/Ya</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>100001</v>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>100001</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>glb</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="2" t="n">
         <v>200001</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Hero/Cube</t>
+      <c r="C5" s="2" t="n"/>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>primitive</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>box</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>800|1600|800</t>
+        </is>
+      </c>
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t>255|140|0|255</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>200002</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>Hero/CubeBlue</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>primitive</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>box</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>800|1600|800</t>
+        </is>
+      </c>
+      <c r="H6" s="0" t="inlineStr">
+        <is>
+          <t>50|128|255|255</t>
         </is>
       </c>
     </row>

</xml_diff>